<commit_message>
Add 'Navigating Cell Addresses' solutions
</commit_message>
<xml_diff>
--- a/navigating-cell-addresses/metro_budget.xlsx
+++ b/navigating-cell-addresses/metro_budget.xlsx
@@ -1,23 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26019"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29711"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary van Valkenburg\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{BAAD70D2-3286-47C7-9C4C-6DF3580ADD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADAF992F-2F25-409B-818D-4B9B36D48F80}"/>
+  <xr:revisionPtr revIDLastSave="140" documentId="13_ncr:1_{BAAD70D2-3286-47C7-9C4C-6DF3580ADD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49B16947-0FF8-430E-AD70-CBBCDBE968F7}"/>
   <bookViews>
-    <workbookView xWindow="135" yWindow="90" windowWidth="21877" windowHeight="13080" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="135" yWindow="90" windowWidth="21877" windowHeight="13080" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metro_budget" sheetId="1" r:id="rId1"/>
     <sheet name="data_dictionary" sheetId="2" r:id="rId2"/>
+    <sheet name="exercises" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="all_departments">metro_budget!$A$2:$A$52</definedName>
+    <definedName name="budget_table">metro_budget!$B$2:$J$52</definedName>
+    <definedName name="metrics">metro_budget!$A$1:$K$1</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -33,8 +42,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="80">
   <si>
     <t>Department</t>
   </si>
@@ -66,6 +97,9 @@
     <t>FY19_diff</t>
   </si>
   <si>
+    <t>Avg_diff</t>
+  </si>
+  <si>
     <t>Administrative</t>
   </si>
   <si>
@@ -247,6 +281,31 @@
   </si>
   <si>
     <t>Actual spending amount - budget amount for fiscal year 2019</t>
+  </si>
+  <si>
+    <t>Questions</t>
+  </si>
+  <si>
+    <t>Review the data dictionary for this dataset.</t>
+  </si>
+  <si>
+    <t>Answers</t>
+  </si>
+  <si>
+    <t>What is the row position for the Sports Authority 2018 Budget amount?</t>
+  </si>
+  <si>
+    <t>What is the column position for the Emergency Communication Center 2019 Actual Spending?</t>
+  </si>
+  <si>
+    <t>Use a formula with ROW() and COLUMN() to find the address of the Mayor’s Office actual spending for 2017.</t>
+  </si>
+  <si>
+    <t>Create a new column at the end of the data called Avg_diff. Find the average difference between each department’s budgeted amount and actual spend amount across all three years. A negative number indicates that the department spent less than budgeted. Copy this formula down to get the average difference for all departments. Do you see a trend?</t>
+  </si>
+  <si>
+    <t>Look for the table shown below at the bottom of the budget spreadsheet. Fill in the cells to report on budget/actual spending differences for select boards and commissions using INDEX() and MATCH(). Bonus: Create and use named regions for the array arguments.
+https://github.com/NewForce-Data-Cohort-12/Data-Curriculum/blob/main/Excel/images/metro_dataset_table.png?raw=true</t>
   </si>
 </sst>
 </file>
@@ -401,7 +460,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -587,6 +646,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -748,11 +813,28 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="135"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="45"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -811,8 +893,25 @@
 </styleSheet>
 </file>
 
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1100,7 +1199,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1108,7 +1207,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
@@ -1120,9 +1219,10 @@
     <col min="7" max="8" width="15.85546875" customWidth="1"/>
     <col min="9" max="9" width="15.42578125" customWidth="1"/>
     <col min="10" max="10" width="17.85546875" customWidth="1"/>
+    <col min="11" max="11" width="31.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1153,10 +1253,13 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>356640100</v>
@@ -1185,10 +1288,14 @@
       <c r="J2">
         <v>-21269107.77</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="K2">
+        <f>AVERAGE(D2,G2,J2)</f>
+        <v>-24336639.273333233</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3">
         <v>328800</v>
@@ -1217,10 +1324,14 @@
       <c r="J3">
         <v>-436.96000000001999</v>
       </c>
-    </row>
-    <row r="4" spans="1:10">
+      <c r="K3">
+        <f t="shared" ref="K3:K52" si="0">AVERAGE(D3,G3,J3)</f>
+        <v>-10129.553333333331</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4">
         <v>3130600</v>
@@ -1249,10 +1360,14 @@
       <c r="J4">
         <v>-97416.950000001103</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="K4">
+        <f t="shared" si="0"/>
+        <v>-58488.72666666747</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B5">
         <v>7670700</v>
@@ -1281,10 +1396,14 @@
       <c r="J5">
         <v>-262277.08999999898</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="K5">
+        <f t="shared" si="0"/>
+        <v>-644371.69999999867</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6">
         <v>409300</v>
@@ -1313,10 +1432,14 @@
       <c r="J6">
         <v>-85.710000000079106</v>
       </c>
-    </row>
-    <row r="7" spans="1:10">
+      <c r="K6">
+        <f t="shared" si="0"/>
+        <v>-8072.8499999999885</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7">
         <v>3329000</v>
@@ -1345,10 +1468,14 @@
       <c r="J7">
         <v>-398759.91999999899</v>
       </c>
-    </row>
-    <row r="8" spans="1:10">
+      <c r="K7">
+        <f t="shared" si="0"/>
+        <v>-373701.76666666596</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8">
         <v>1552100</v>
@@ -1377,10 +1504,14 @@
       <c r="J8">
         <v>-241564.68</v>
       </c>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="K8">
+        <f t="shared" si="0"/>
+        <v>-228278.46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B9">
         <v>9349400</v>
@@ -1409,74 +1540,86 @@
       <c r="J9">
         <v>-796900.47000000405</v>
       </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10">
+      <c r="K9">
+        <f t="shared" si="0"/>
+        <v>-779371.89000000141</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" s="8" customFormat="1">
+      <c r="A10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="8">
         <v>443300</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="8">
         <v>407090.37</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="8">
         <v>-36209.629999999903</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="8">
         <v>495200</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="8">
         <v>467907.84000000003</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="8">
         <v>-27292.159999999902</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="8">
         <v>487500</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="8">
         <v>478318.92</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="8">
         <v>-9181.0800000000108</v>
       </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11">
-        <v>0</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
+      <c r="K10" s="8">
+        <f t="shared" si="0"/>
+        <v>-24227.623333333275</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" s="8" customFormat="1">
+      <c r="A11" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="8">
+        <v>0</v>
+      </c>
+      <c r="C11" s="8">
+        <v>0</v>
+      </c>
+      <c r="D11" s="8">
+        <v>0</v>
+      </c>
+      <c r="E11" s="8">
+        <v>0</v>
+      </c>
+      <c r="F11" s="8">
+        <v>0</v>
+      </c>
+      <c r="G11" s="8">
+        <v>0</v>
+      </c>
+      <c r="H11" s="8">
         <v>375000</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="8">
         <v>63771.91</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="8">
         <v>-311228.08999999898</v>
       </c>
-    </row>
-    <row r="12" spans="1:10">
+      <c r="K11" s="8">
+        <f t="shared" si="0"/>
+        <v>-103742.69666666632</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B12">
         <v>4280900</v>
@@ -1505,10 +1648,14 @@
       <c r="J12">
         <v>-306086.86</v>
       </c>
-    </row>
-    <row r="13" spans="1:10">
+      <c r="K12">
+        <f t="shared" si="0"/>
+        <v>-338411.97666666534</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13">
         <v>5847800</v>
@@ -1537,10 +1684,14 @@
       <c r="J13">
         <v>-150323.329999999</v>
       </c>
-    </row>
-    <row r="14" spans="1:10">
+      <c r="K13">
+        <f t="shared" si="0"/>
+        <v>-180152.35333333295</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B14">
         <v>512000</v>
@@ -1569,10 +1720,14 @@
       <c r="J14">
         <v>-21210.119999999901</v>
       </c>
-    </row>
-    <row r="15" spans="1:10">
+      <c r="K14">
+        <f t="shared" si="0"/>
+        <v>-11429.923333333229</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15">
         <v>156049100</v>
@@ -1601,10 +1756,14 @@
       <c r="J15">
         <v>-4502589.1500000302</v>
       </c>
-    </row>
-    <row r="16" spans="1:10">
+      <c r="K15">
+        <f t="shared" si="0"/>
+        <v>-4069060.0000000186</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16">
         <v>6600700</v>
@@ -1633,10 +1792,14 @@
       <c r="J16">
         <v>-106.999999999068</v>
       </c>
-    </row>
-    <row r="17" spans="1:10">
+      <c r="K16">
+        <f t="shared" si="0"/>
+        <v>-26787.486666666631</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B17">
         <v>14860800</v>
@@ -1665,42 +1828,50 @@
       <c r="J17">
         <v>-965742.96</v>
       </c>
-    </row>
-    <row r="18" spans="1:10">
-      <c r="A18" t="s">
-        <v>26</v>
-      </c>
-      <c r="B18">
+      <c r="K17">
+        <f t="shared" si="0"/>
+        <v>-683843.13333333295</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" s="8" customFormat="1">
+      <c r="A18" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="8">
         <v>2764700</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="8">
         <v>2615303.8999999901</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="8">
         <v>-149396.1</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="8">
         <v>2861000</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="8">
         <v>2671745.94</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="8">
         <v>-189254.05999999901</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="8">
         <v>2910600</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="8">
         <v>2535637.09</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="8">
         <v>-374962.91</v>
       </c>
-    </row>
-    <row r="19" spans="1:10">
+      <c r="K18" s="8">
+        <f t="shared" si="0"/>
+        <v>-237871.02333333297</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19">
         <v>8837300</v>
@@ -1729,10 +1900,14 @@
       <c r="J19">
         <v>-576344.08999999403</v>
       </c>
-    </row>
-    <row r="20" spans="1:10">
+      <c r="K19">
+        <f t="shared" si="0"/>
+        <v>-558091.21666666702</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B20">
         <v>124385900</v>
@@ -1761,10 +1936,14 @@
       <c r="J20">
         <v>-116.46000003814601</v>
       </c>
-    </row>
-    <row r="21" spans="1:10">
+      <c r="K20">
+        <f t="shared" si="0"/>
+        <v>-3810.6433333406817</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B21">
         <v>24332100</v>
@@ -1793,10 +1972,14 @@
       <c r="J21">
         <v>-888926.91000000294</v>
       </c>
-    </row>
-    <row r="22" spans="1:10">
+      <c r="K21">
+        <f t="shared" si="0"/>
+        <v>-1551281.9100000076</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B22">
         <v>11566000</v>
@@ -1825,10 +2008,14 @@
       <c r="J22">
         <v>-745.22999999672095</v>
       </c>
-    </row>
-    <row r="23" spans="1:10">
+      <c r="K22">
+        <f t="shared" si="0"/>
+        <v>-114375.79333333323</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B23">
         <v>20862700</v>
@@ -1857,74 +2044,86 @@
       <c r="J23">
         <v>-601242.55999998702</v>
       </c>
-    </row>
-    <row r="24" spans="1:10">
-      <c r="A24" t="s">
-        <v>32</v>
-      </c>
-      <c r="B24">
+      <c r="K23">
+        <f t="shared" si="0"/>
+        <v>-796290.97666667739</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" s="8" customFormat="1">
+      <c r="A24" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="8">
         <v>917200</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="8">
         <v>904969.19</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="8">
         <v>-12230.809999999799</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="8">
         <v>1112700</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="8">
         <v>1067214.42</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="8">
         <v>-45485.579999999798</v>
       </c>
-      <c r="H24">
+      <c r="H24" s="8">
         <v>1112600</v>
       </c>
-      <c r="I24">
+      <c r="I24" s="8">
         <v>1112527.1200000001</v>
       </c>
-      <c r="J24">
+      <c r="J24" s="8">
         <v>-72.879999999888199</v>
       </c>
-    </row>
-    <row r="25" spans="1:10">
-      <c r="A25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25">
+      <c r="K24" s="8">
+        <f t="shared" si="0"/>
+        <v>-19263.089999999829</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" s="8" customFormat="1">
+      <c r="A25" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="8">
         <v>484100</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="8">
         <v>479149.53</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="8">
         <v>-4950.4699999999102</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="8">
         <v>505200</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="8">
         <v>497194.20999999897</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="8">
         <v>-8005.79000000003</v>
       </c>
-      <c r="H25">
+      <c r="H25" s="8">
         <v>496500</v>
       </c>
-      <c r="I25">
+      <c r="I25" s="8">
         <v>494775.1</v>
       </c>
-      <c r="J25">
+      <c r="J25" s="8">
         <v>-1724.8999999999601</v>
       </c>
-    </row>
-    <row r="26" spans="1:10">
+      <c r="K25" s="8">
+        <f t="shared" si="0"/>
+        <v>-4893.7199999999666</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B26">
         <v>5249800</v>
@@ -1953,10 +2152,14 @@
       <c r="J26">
         <v>-313464.78999999998</v>
       </c>
-    </row>
-    <row r="27" spans="1:10">
+      <c r="K26">
+        <f t="shared" si="0"/>
+        <v>-360391.89333333302</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -1985,10 +2188,14 @@
       <c r="J27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:10">
+      <c r="K27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B28">
         <v>1382900</v>
@@ -2017,10 +2224,14 @@
       <c r="J28">
         <v>-132614.93999999901</v>
       </c>
-    </row>
-    <row r="29" spans="1:10">
+      <c r="K28">
+        <f t="shared" si="0"/>
+        <v>-176479.22999999937</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B29">
         <v>2561800</v>
@@ -2049,10 +2260,14 @@
       <c r="J29">
         <v>-35.329999999143098</v>
       </c>
-    </row>
-    <row r="30" spans="1:10">
+      <c r="K29">
+        <f t="shared" si="0"/>
+        <v>-50728.72666666608</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B30">
         <v>12132200</v>
@@ -2081,10 +2296,14 @@
       <c r="J30">
         <v>-35290.389999991203</v>
       </c>
-    </row>
-    <row r="31" spans="1:10">
+      <c r="K30">
+        <f t="shared" si="0"/>
+        <v>-62460.669999994228</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B31">
         <v>1765600</v>
@@ -2113,10 +2332,14 @@
       <c r="J31">
         <v>-69308.659999999596</v>
       </c>
-    </row>
-    <row r="32" spans="1:10">
+      <c r="K31">
+        <f t="shared" si="0"/>
+        <v>-51568.039999999601</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B32">
         <v>5999400</v>
@@ -2145,10 +2368,14 @@
       <c r="J32">
         <v>-169827.98</v>
       </c>
-    </row>
-    <row r="33" spans="1:10">
+      <c r="K32">
+        <f t="shared" si="0"/>
+        <v>-118034.93000000005</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B33">
         <v>927703099.99999905</v>
@@ -2177,10 +2404,14 @@
       <c r="J33">
         <v>-5456610.5900001498</v>
       </c>
-    </row>
-    <row r="34" spans="1:10">
+      <c r="K33">
+        <f t="shared" si="0"/>
+        <v>-5159310.7933333265</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B34">
         <v>4189300</v>
@@ -2209,10 +2440,14 @@
       <c r="J34">
         <v>-115798.49</v>
       </c>
-    </row>
-    <row r="35" spans="1:10">
+      <c r="K34">
+        <f t="shared" si="0"/>
+        <v>-136050.49999999962</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B35">
         <v>0</v>
@@ -2241,10 +2476,14 @@
       <c r="J35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:10">
+      <c r="K35">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B36">
         <v>798200</v>
@@ -2273,10 +2512,14 @@
       <c r="J36">
         <v>-101084.71</v>
       </c>
-    </row>
-    <row r="37" spans="1:10">
+      <c r="K36">
+        <f t="shared" si="0"/>
+        <v>-107198.16000000008</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B37">
         <v>2087800</v>
@@ -2305,10 +2548,14 @@
       <c r="J37">
         <v>-188181.66</v>
       </c>
-    </row>
-    <row r="38" spans="1:10">
+      <c r="K37">
+        <f t="shared" si="0"/>
+        <v>-126930.23666666658</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B38">
         <v>855300</v>
@@ -2337,10 +2584,14 @@
       <c r="J38">
         <v>-136.73999999987399</v>
       </c>
-    </row>
-    <row r="39" spans="1:10">
+      <c r="K38">
+        <f t="shared" si="0"/>
+        <v>-18704.986666666489</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B39">
         <v>883900</v>
@@ -2369,10 +2620,14 @@
       <c r="J39">
         <v>-79036.130000000296</v>
       </c>
-    </row>
-    <row r="40" spans="1:10">
+      <c r="K39">
+        <f t="shared" si="0"/>
+        <v>-109994.99333333345</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B40">
         <v>38381900</v>
@@ -2401,42 +2656,50 @@
       <c r="J40">
         <v>-610436.29000002099</v>
       </c>
-    </row>
-    <row r="41" spans="1:10">
-      <c r="A41" t="s">
-        <v>49</v>
-      </c>
-      <c r="B41">
+      <c r="K40">
+        <f t="shared" si="0"/>
+        <v>-1098951.4133333552</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" s="8" customFormat="1">
+      <c r="A41" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" s="8">
         <v>4593300</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="8">
         <v>4409060.2099999897</v>
       </c>
-      <c r="D41">
+      <c r="D41" s="8">
         <v>-184239.79</v>
       </c>
-      <c r="E41">
+      <c r="E41" s="8">
         <v>5089500</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="8">
         <v>4956043.6699999897</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="8">
         <v>-133456.33000000101</v>
       </c>
-      <c r="H41">
+      <c r="H41" s="8">
         <v>4799900</v>
       </c>
-      <c r="I41">
+      <c r="I41" s="8">
         <v>4717822.6500000004</v>
       </c>
-      <c r="J41">
+      <c r="J41" s="8">
         <v>-82077.349999997707</v>
       </c>
-    </row>
-    <row r="42" spans="1:10">
+      <c r="K41" s="8">
+        <f t="shared" si="0"/>
+        <v>-133257.82333333293</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B42">
         <v>188593300</v>
@@ -2465,10 +2728,14 @@
       <c r="J42">
         <v>-36.250000059604602</v>
       </c>
-    </row>
-    <row r="43" spans="1:10">
+      <c r="K42">
+        <f t="shared" si="0"/>
+        <v>-805642.42000006372</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11">
       <c r="A43" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B43">
         <v>8135400</v>
@@ -2497,10 +2764,14 @@
       <c r="J43">
         <v>-346517.43</v>
       </c>
-    </row>
-    <row r="44" spans="1:10">
+      <c r="K43">
+        <f t="shared" si="0"/>
+        <v>-300866.52666666568</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11">
       <c r="A44" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B44">
         <v>30083200</v>
@@ -2529,10 +2800,14 @@
       <c r="J44">
         <v>-58.749999988824101</v>
       </c>
-    </row>
-    <row r="45" spans="1:10">
+      <c r="K44">
+        <f t="shared" si="0"/>
+        <v>-180380.9633333206</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11">
       <c r="A45" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B45">
         <v>55301600</v>
@@ -2561,10 +2836,14 @@
       <c r="J45">
         <v>-640550.34000001801</v>
       </c>
-    </row>
-    <row r="46" spans="1:10">
+      <c r="K45">
+        <f t="shared" si="0"/>
+        <v>-1183270.7766666792</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11">
       <c r="A46" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B46">
         <v>259100</v>
@@ -2593,10 +2872,14 @@
       <c r="J46">
         <v>-12346.84</v>
       </c>
-    </row>
-    <row r="47" spans="1:10">
+      <c r="K46">
+        <f t="shared" si="0"/>
+        <v>-7240.50000000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11">
       <c r="A47" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B47">
         <v>70390700</v>
@@ -2625,10 +2908,14 @@
       <c r="J47">
         <v>-21970.8200000822</v>
       </c>
-    </row>
-    <row r="48" spans="1:10">
+      <c r="K47">
+        <f t="shared" si="0"/>
+        <v>-19567.480000009065</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11">
       <c r="A48" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B48">
         <v>6737100</v>
@@ -2657,10 +2944,14 @@
       <c r="J48">
         <v>-407449.76000000199</v>
       </c>
-    </row>
-    <row r="49" spans="1:10">
+      <c r="K48">
+        <f t="shared" si="0"/>
+        <v>-303274.87666666665</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11">
       <c r="A49" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B49">
         <v>92200</v>
@@ -2689,10 +2980,14 @@
       <c r="J49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:10">
+      <c r="K49">
+        <f t="shared" si="0"/>
+        <v>-2944.563333333323</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11">
       <c r="A50" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B50">
         <v>832600</v>
@@ -2721,10 +3016,14 @@
       <c r="J50">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:10">
+      <c r="K50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11">
       <c r="A51" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B51">
         <v>8609500</v>
@@ -2753,10 +3052,14 @@
       <c r="J51">
         <v>-98056.689999999406</v>
       </c>
-    </row>
-    <row r="52" spans="1:10">
+      <c r="K51">
+        <f t="shared" si="0"/>
+        <v>-178190.57666666713</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="15">
       <c r="A52" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B52">
         <v>2451000</v>
@@ -2785,8 +3088,12 @@
       <c r="J52">
         <v>-264764.74</v>
       </c>
-    </row>
-    <row r="55" spans="1:10">
+      <c r="K52">
+        <f t="shared" si="0"/>
+        <v>-232369.01999999932</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11">
       <c r="A55" s="1" t="s">
         <v>0</v>
       </c>
@@ -2800,34 +3107,106 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:10">
+    <row r="56" spans="1:11" ht="15">
       <c r="A56" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10">
+        <v>19</v>
+      </c>
+      <c r="B56" s="4" cm="1">
+        <f t="array" ref="B56">INDEX(budget_table,MATCH($A56,all_departments,0),MATCH(B$55,metrics,0)-1)</f>
+        <v>-36209.629999999903</v>
+      </c>
+      <c r="C56" s="4" cm="1">
+        <f t="array" ref="C56">INDEX(budget_table,MATCH($A56,all_departments,0),MATCH(C$55,metrics,0)-1)</f>
+        <v>-27292.159999999902</v>
+      </c>
+      <c r="D56" s="4" cm="1">
+        <f t="array" ref="D56">INDEX(budget_table,MATCH($A56,all_departments,0),MATCH(D$55,metrics,0)-1)</f>
+        <v>-9181.0800000000108</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="15">
       <c r="A57" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10">
+        <v>20</v>
+      </c>
+      <c r="B57" s="4" cm="1">
+        <f t="array" ref="B57">INDEX(budget_table,MATCH($A57,all_departments,0),MATCH(B$55,metrics,0)-1)</f>
+        <v>0</v>
+      </c>
+      <c r="C57" s="4" cm="1">
+        <f t="array" ref="C57">INDEX(budget_table,MATCH($A57,all_departments,0),MATCH(C$55,metrics,0)-1)</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="4" cm="1">
+        <f t="array" ref="D57">INDEX(budget_table,MATCH($A57,all_departments,0),MATCH(D$55,metrics,0)-1)</f>
+        <v>-311228.08999999898</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="15">
       <c r="A58" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10">
+        <v>27</v>
+      </c>
+      <c r="B58" s="4" cm="1">
+        <f t="array" ref="B58">INDEX(budget_table,MATCH($A58,all_departments,0),MATCH(B$55,metrics,0)-1)</f>
+        <v>-149396.1</v>
+      </c>
+      <c r="C58" s="4" cm="1">
+        <f t="array" ref="C58">INDEX(budget_table,MATCH($A58,all_departments,0),MATCH(C$55,metrics,0)-1)</f>
+        <v>-189254.05999999901</v>
+      </c>
+      <c r="D58" s="4" cm="1">
+        <f t="array" ref="D58">INDEX(budget_table,MATCH($A58,all_departments,0),MATCH(D$55,metrics,0)-1)</f>
+        <v>-374962.91</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="15">
       <c r="A59" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10">
+        <v>33</v>
+      </c>
+      <c r="B59" s="4" cm="1">
+        <f t="array" ref="B59">INDEX(budget_table,MATCH($A59,all_departments,0),MATCH(B$55,metrics,0)-1)</f>
+        <v>-12230.809999999799</v>
+      </c>
+      <c r="C59" s="4" cm="1">
+        <f t="array" ref="C59">INDEX(budget_table,MATCH($A59,all_departments,0),MATCH(C$55,metrics,0)-1)</f>
+        <v>-45485.579999999798</v>
+      </c>
+      <c r="D59" s="4" cm="1">
+        <f t="array" ref="D59">INDEX(budget_table,MATCH($A59,all_departments,0),MATCH(D$55,metrics,0)-1)</f>
+        <v>-72.879999999888199</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="15">
       <c r="A60" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10">
+        <v>34</v>
+      </c>
+      <c r="B60" s="4" cm="1">
+        <f t="array" ref="B60">INDEX(budget_table,MATCH($A60,all_departments,0),MATCH(B$55,metrics,0)-1)</f>
+        <v>-4950.4699999999102</v>
+      </c>
+      <c r="C60" s="4" cm="1">
+        <f t="array" ref="C60">INDEX(budget_table,MATCH($A60,all_departments,0),MATCH(C$55,metrics,0)-1)</f>
+        <v>-8005.79000000003</v>
+      </c>
+      <c r="D60" s="4" cm="1">
+        <f t="array" ref="D60">INDEX(budget_table,MATCH($A60,all_departments,0),MATCH(D$55,metrics,0)-1)</f>
+        <v>-1724.8999999999601</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="15">
       <c r="A61" t="s">
-        <v>49</v>
+        <v>50</v>
+      </c>
+      <c r="B61" s="4" cm="1">
+        <f t="array" ref="B61">INDEX(budget_table,MATCH($A61,all_departments,0),MATCH(B$55,metrics,0)-1)</f>
+        <v>-184239.79</v>
+      </c>
+      <c r="C61" s="4" cm="1">
+        <f t="array" ref="C61">INDEX(budget_table,MATCH($A61,all_departments,0),MATCH(C$55,metrics,0)-1)</f>
+        <v>-133456.33000000101</v>
+      </c>
+      <c r="D61" s="4" cm="1">
+        <f t="array" ref="D61">INDEX(budget_table,MATCH($A61,all_departments,0),MATCH(D$55,metrics,0)-1)</f>
+        <v>-82077.349999997707</v>
       </c>
     </row>
   </sheetData>
@@ -2849,7 +3228,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -2857,7 +3236,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -2865,7 +3244,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -2873,7 +3252,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2881,7 +3260,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -2889,7 +3268,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -2897,7 +3276,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -2905,7 +3284,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2913,7 +3292,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -2921,10 +3300,106 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF70C7AD-43A8-45C4-AB9E-227CE7DC62C9}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="30.75">
+      <c r="A1" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="30.75">
+      <c r="A2" s="6"/>
+      <c r="B2" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2">
+        <f>MATCH("Sports Authority",metro_budget!$A$1:$A$52,0)</f>
+        <v>50</v>
+      </c>
+      <c r="D2" s="7"/>
+      <c r="E2">
+        <f>MATCH("FY18_Budget",metro_budget!$A$1:$J$1)</f>
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <f>MATCH("Sports Authority",metro_budget!$A$1:$A$52)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="45.75">
+      <c r="A3" s="6"/>
+      <c r="B3" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3">
+        <f>MATCH("FY19_Actual",metro_budget!$A$1:$J$1,0)</f>
+        <v>9</v>
+      </c>
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" spans="1:6" ht="45.75">
+      <c r="A4" s="6"/>
+      <c r="B4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="4" t="str">
+        <f>CONCATENATE("[R=",ROW($C$34),"][C=",COLUMN($C$34),"]")</f>
+        <v>[R=34][C=3]</v>
+      </c>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:6" ht="152.25">
+      <c r="A5" s="6"/>
+      <c r="B5" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5">
+        <f>AVERAGE(metro_budget!D2,metro_budget!G2,metro_budget!J2)</f>
+        <v>-24336639.273333233</v>
+      </c>
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:6" ht="167.25">
+      <c r="A6" s="6"/>
+      <c r="B6" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" cm="1">
+        <f t="array" ref="C6">INDEX(budget_table,MATCH(metro_budget!$A56,all_departments,0),MATCH(metro_budget!B$55,metrics,0)-1)</f>
+        <v>-36209.629999999903</v>
+      </c>
+      <c r="D6" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:A6"/>
+    <mergeCell ref="D1:D6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>